<commit_message>
Update Production Master: Cohort 1 Batch A Supabase entry complete
Set Supabase Status=Complete, Enc Production Status=Full Entry Live,
Research Status=Complete, Canonical MD Status=Approved for:
Amazonite, Amethyst, Black Tourmaline, Carnelian, Clear Quartz, Green Aventurine

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/encyclopedia/production-data/Still-Point-Lapidary-Production-Master.xlsx
+++ b/docs/encyclopedia/production-data/Still-Point-Lapidary-Production-Master.xlsx
@@ -736,7 +736,7 @@
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>MD Approved</t>
+          <t>Full Entry Live</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -839,7 +839,7 @@
       </c>
       <c r="AO2" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="AP2" t="inlineStr">
@@ -931,7 +931,7 @@
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>MD Approved</t>
+          <t>Full Entry Live</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
@@ -1024,7 +1024,7 @@
       </c>
       <c r="AO3" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="AP3" t="inlineStr">
@@ -1111,7 +1111,7 @@
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>MD Approved</t>
+          <t>Full Entry Live</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
@@ -1209,7 +1209,7 @@
       </c>
       <c r="AO4" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="AP4" t="inlineStr">
@@ -1481,7 +1481,7 @@
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>MD Approved</t>
+          <t>Full Entry Live</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
@@ -1574,7 +1574,7 @@
       </c>
       <c r="AO6" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="AP6" t="inlineStr">
@@ -1661,7 +1661,7 @@
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>MD Approved</t>
+          <t>Full Entry Live</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
@@ -1754,7 +1754,7 @@
       </c>
       <c r="AO7" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="AP7" t="inlineStr">
@@ -3976,7 +3976,7 @@
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>MD Approved</t>
+          <t>Full Entry Live</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
@@ -4074,7 +4074,7 @@
       </c>
       <c r="AO22" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="AP22" t="inlineStr">

</xml_diff>

<commit_message>
Update Production Master: Amethyst chakra correction
Primary Chakra = Third Eye, Secondary Chakra = Crown
Aligns with approved canonical MD.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/encyclopedia/production-data/Still-Point-Lapidary-Production-Master.xlsx
+++ b/docs/encyclopedia/production-data/Still-Point-Lapidary-Production-Master.xlsx
@@ -741,12 +741,12 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
+          <t>Third Eye</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
           <t>Crown</t>
-        </is>
-      </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>Third Eye</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">

</xml_diff>